<commit_message>
Simple Flow: SV-8183 vs QA-issues analysis + corrective lesson (report over-claimed; 3 coverage gaps)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/simple-flow/sv8183/SimpleFlow_SV-8183_Permission-Test-Report_2026-07-23.xlsx
+++ b/build/simple-flow/sv8183/SimpleFlow_SV-8183_Permission-Test-Report_2026-07-23.xlsx
@@ -23,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -58,8 +58,17 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -84,6 +93,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -113,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -143,6 +157,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -510,91 +530,138 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="118" customWidth="1" min="1" max="1"/>
+    <col width="120" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>⚠️ CORRECTION 2026-07-24 — this report OVER-CLAIMED completeness (read first).</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="14" t="inlineStr">
+        <is>
+          <t>This report concluded "11/11 PASS, controls behave exactly as specified." That was over-claimed. QA (Ayesha) then raised SV-8515, SV-8516, SV-8541; a live re-verify on clean template roles (2026-07-24) confirmed all three are REAL coverage gaps.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="14" t="inlineStr">
+        <is>
+          <t>SV-8515: real front-end-exposure defect (dev Ready-to-Fix) — View-only user can multi-select "Receive Selected" to the editable Bulk-Receive screen; actual receive blocked at back end (accept → 403), so a misleading dead-end, NOT a data bypass.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>SV-8516: real over-grant, front-end now FIXED (Time Clock ⋮ = only Return), but back end still accepts a part edit (change-request → 200) = Rule-24 API flag.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="64" customHeight="1">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>SV-8541: real; role without WO Lines: Create &amp; Edit can resolve cores (pre-resolve-cores → 201, even Time Clock); pre-existing (matches Production), §9.4-anticipated, Open for Sasha.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>The 11 cases still pass for what they tested; the feature-wide PASS below is CORRECTED to a SCOPED pass. Full analysis + 3 proposed corrective cases: SimpleFlow_SV-8183_vs-QA-Issues_Analysis_2026-07-24.md/.xlsx (same folder).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="64" customHeight="1">
+      <c r="A8" s="1" t="inlineStr">
         <is>
           <t>Simple Flow — SV-8183 Permission Test: Management Report</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Date tested 2026-07-23  ·  Environment: live staging (app.staging.shopview.com)  ·  Product Owner: Milos  ·  No TestRail results written</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+    <row r="10"/>
+    <row r="11" ht="64" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>What this is.</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="64" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Every ShopView user has a role (Admin, Service Advisor, Technician, Office, etc.). A role decides which buttons and screens that person can use. SV-8183 defines, for the new Simple Flow feature, exactly which roles may do each action — finish a work order, sign it off, order parts, change settings, and so on. This report is the result of testing those role controls on the real system.</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+    <row r="13"/>
+    <row r="14" ht="64" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>What "testing the permissions" means, plainly.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="64" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>For each action we asked two simple questions: (1) Do the right people have it, and the wrong people not have it? and (2) Does the system actually stop the wrong people? We answered both by logging in as each role on the live staging system and looking at the real screens and buttons, with screenshots as proof. We did NOT guess from documents or code.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+    <row r="16"/>
+    <row r="17" ht="64" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>How we made the test fair.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="64" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Before testing, every role was reset to its correct default set of permissions, so we tested the intended rules and not leftover changes from other testers. We confirmed all 11 roles were already at their correct defaults.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+    <row r="19"/>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>Headline result.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="64" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>We checked 10 core permissions across all 11 roles (that is 110 role-and-permission combinations), backed by 11 formal test cases. Every combination matched the specification exactly — zero mismatches — and all 11 test cases passed (11 passed, 0 failed, 0 blocked). The system correctly gives each role only the actions it should have and blocks the rest, both on the screen and (where tested) in the underlying system.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+    <row r="22"/>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>Verdict: PASS.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="64" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>Simple Flow's role and permission controls behave exactly as specified — the right roles can do each action and the wrong roles are blocked — with one design point noted for clarity (see the Findings tab), which is not a failure.</t>
         </is>

</xml_diff>